<commit_message>
Refine point scale to six levels and drop external-division item
배점을 하3·중하4·중5·중상6·상7·최상8로 세분화하고 객관식 최고 배점을
7점으로 제한(과목별 100점 유지). 공통수학2 18번의 외분점 문항을 내분점으로
점 P를 정하는 거리 최대·최소 문항으로 교체. 시험지·미리보기·채점 엑셀
재생성, 40문항 정답 재검증.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="176">
   <si>
     <r>
       <rPr>
@@ -3513,7 +3513,13 @@
     <t xml:space="preserve">하</t>
   </si>
   <si>
+    <t xml:space="preserve">중하</t>
+  </si>
+  <si>
     <t xml:space="preserve">중</t>
+  </si>
+  <si>
+    <t xml:space="preserve">중상</t>
   </si>
   <si>
     <t xml:space="preserve">상</t>
@@ -5830,7 +5836,7 @@
       </c>
       <c r="D19" s="10" t="n">
         <f aca="false">SUMIF(공수1!$D$4:$W$4,B19,공수1!$D$3:$W$3)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>31</v>
@@ -5849,7 +5855,7 @@
       </c>
       <c r="D20" s="10" t="n">
         <f aca="false">SUMIF(공수1!$D$4:$W$4,B20,공수1!$D$3:$W$3)</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -5887,7 +5893,7 @@
       </c>
       <c r="D22" s="10" t="n">
         <f aca="false">SUMIF(공수1!$D$4:$W$4,B22,공수1!$D$3:$W$3)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>37</v>
@@ -5925,7 +5931,7 @@
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">SUMIF(공수2!$D$4:$W$4,B24,공수2!$D$3:$W$3)</f>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>42</v>
@@ -5963,7 +5969,7 @@
       </c>
       <c r="D26" s="10" t="n">
         <f aca="false">SUMIF(공수2!$D$4:$W$4,B26,공수2!$D$3:$W$3)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>46</v>
@@ -7414,13 +7420,13 @@
         <v>3</v>
       </c>
       <c r="G3" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" s="20" t="n">
         <v>5</v>
@@ -7429,7 +7435,7 @@
         <v>5</v>
       </c>
       <c r="L3" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M3" s="20" t="n">
         <v>6</v>
@@ -7438,19 +7444,19 @@
         <v>6</v>
       </c>
       <c r="O3" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P3" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q3" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R3" s="20" t="n">
         <v>3</v>
       </c>
       <c r="S3" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T3" s="20" t="n">
         <v>5</v>
@@ -7474,11 +7480,11 @@
       </c>
       <c r="Z3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,Z$6,$D$3:$W$3)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AA3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,AA$6,$D$3:$W$3)</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AB3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,AB$6,$D$3:$W$3)</f>
@@ -7486,7 +7492,7 @@
       </c>
       <c r="AC3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,AC$6,$D$3:$W$3)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7572,7 +7578,7 @@
         <v>101</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>102</v>
@@ -7581,64 +7587,64 @@
         <v>102</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>103</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="R5" s="6" t="s">
         <v>101</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="X5" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Y5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="Z5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AA5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AB5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AC5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7652,70 +7658,70 @@
         <v>84</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I6" s="28" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J6" s="28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O6" s="28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P6" s="28" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="Q6" s="28" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="R6" s="29" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="S6" s="29" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="T6" s="29" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="U6" s="29" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="V6" s="29" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="W6" s="29" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="Z6" s="30" t="str">
         <f aca="false">설정!B19</f>
@@ -12314,14 +12320,6 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
-      <formula1>설정!$B$19:$B$22</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
-      <formula1>"하,중,상,최상"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -12329,6 +12327,14 @@
     <dataValidation allowBlank="true" error="단답형은 0~999 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R2:W2 R7:W86" type="whole">
       <formula1>0</formula1>
       <formula2>999</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
+      <formula1>설정!$B$19:$B$22</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
+      <formula1>"하,중하,중,중상,상,최상"</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12360,7 +12366,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12475,13 +12481,13 @@
         <v>3</v>
       </c>
       <c r="G3" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" s="20" t="n">
         <v>5</v>
@@ -12490,7 +12496,7 @@
         <v>5</v>
       </c>
       <c r="L3" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M3" s="20" t="n">
         <v>6</v>
@@ -12499,19 +12505,19 @@
         <v>6</v>
       </c>
       <c r="O3" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P3" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q3" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R3" s="20" t="n">
         <v>3</v>
       </c>
       <c r="S3" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T3" s="20" t="n">
         <v>5</v>
@@ -12535,7 +12541,7 @@
       </c>
       <c r="Z3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,Z$6,$D$3:$W$3)</f>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AA3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,AA$6,$D$3:$W$3)</f>
@@ -12543,7 +12549,7 @@
       </c>
       <c r="AB3" s="18" t="n">
         <f aca="false">SUMIF($D$4:$W$4,AB$6,$D$3:$W$3)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12629,7 +12635,7 @@
         <v>101</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>102</v>
@@ -12638,61 +12644,61 @@
         <v>102</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>103</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="R5" s="6" t="s">
         <v>101</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="X5" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Y5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="Z5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AA5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AB5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12706,70 +12712,70 @@
         <v>84</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I6" s="28" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J6" s="28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O6" s="28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P6" s="28" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="Q6" s="28" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="R6" s="29" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="S6" s="29" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="T6" s="29" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="U6" s="29" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="V6" s="29" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="W6" s="29" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="Z6" s="30" t="str">
         <f aca="false">설정!B24</f>
@@ -17044,6 +17050,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
+      <formula1>설정!$B$24:$B$26</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
+      <formula1>"하,중하,중,중상,상,최상"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -17051,14 +17065,6 @@
     <dataValidation allowBlank="true" error="단답형은 0~999 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R2:W2 R7:W86" type="whole">
       <formula1>0</formula1>
       <formula2>999</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
-      <formula1>설정!$B$24:$B$26</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
-      <formula1>"하,중,상,최상"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -17096,7 +17102,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17121,7 +17127,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -17146,7 +17152,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P5" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17163,55 +17169,55 @@
         <v>85</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="W6" s="4" t="s">
         <v>91</v>
@@ -17665,7 +17671,7 @@
         <v/>
       </c>
       <c r="P12" s="22" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="Q12" s="22"/>
       <c r="R12" s="22"/>
@@ -21745,7 +21751,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -21759,7 +21765,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -21773,7 +21779,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>83</v>
@@ -21785,22 +21791,22 @@
         <v>85</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H6" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I6" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="J6" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25852,7 +25858,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -25874,7 +25880,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -25896,7 +25902,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="42" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" s="42"/>
       <c r="C4" s="42"/>
@@ -25905,31 +25911,31 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -25944,25 +25950,25 @@
         <v>기본반 정답률</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O5" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P5" s="19" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R5" s="19" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25970,7 +25976,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C6" s="43" t="str">
         <f aca="false">공수1!D4</f>
@@ -26046,7 +26052,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C7" s="43" t="str">
         <f aca="false">공수1!E4</f>
@@ -26122,7 +26128,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C8" s="43" t="str">
         <f aca="false">공수1!F4</f>
@@ -26198,7 +26204,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C9" s="43" t="str">
         <f aca="false">공수1!G4</f>
@@ -26206,11 +26212,11 @@
       </c>
       <c r="D9" s="10" t="str">
         <f aca="false">공수1!G5</f>
-        <v>하</v>
+        <v>중하</v>
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">공수1!G3</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="44" t="n">
         <f aca="false">IF(공수1!$G$2="","",공수1!$G$2)</f>
@@ -26274,7 +26280,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C10" s="43" t="str">
         <f aca="false">공수1!H4</f>
@@ -26282,11 +26288,11 @@
       </c>
       <c r="D10" s="10" t="str">
         <f aca="false">공수1!H5</f>
-        <v>중</v>
+        <v>중하</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">공수1!H3</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="44" t="n">
         <f aca="false">IF(공수1!$H$2="","",공수1!$H$2)</f>
@@ -26350,7 +26356,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C11" s="43" t="str">
         <f aca="false">공수1!I4</f>
@@ -26358,11 +26364,11 @@
       </c>
       <c r="D11" s="10" t="str">
         <f aca="false">공수1!I5</f>
-        <v>중</v>
+        <v>중하</v>
       </c>
       <c r="E11" s="10" t="n">
         <f aca="false">공수1!I3</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" s="44" t="n">
         <f aca="false">IF(공수1!$I$2="","",공수1!$I$2)</f>
@@ -26426,7 +26432,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C12" s="43" t="str">
         <f aca="false">공수1!J4</f>
@@ -26502,7 +26508,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C13" s="43" t="str">
         <f aca="false">공수1!K4</f>
@@ -26578,7 +26584,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C14" s="43" t="str">
         <f aca="false">공수1!L4</f>
@@ -26586,11 +26592,11 @@
       </c>
       <c r="D14" s="10" t="str">
         <f aca="false">공수1!L5</f>
-        <v>상</v>
+        <v>중</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">공수1!L3</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F14" s="44" t="n">
         <f aca="false">IF(공수1!$L$2="","",공수1!$L$2)</f>
@@ -26654,7 +26660,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C15" s="43" t="str">
         <f aca="false">공수1!M4</f>
@@ -26662,7 +26668,7 @@
       </c>
       <c r="D15" s="10" t="str">
         <f aca="false">공수1!M5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E15" s="10" t="n">
         <f aca="false">공수1!M3</f>
@@ -26730,7 +26736,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C16" s="43" t="str">
         <f aca="false">공수1!N4</f>
@@ -26738,7 +26744,7 @@
       </c>
       <c r="D16" s="10" t="str">
         <f aca="false">공수1!N5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E16" s="10" t="n">
         <f aca="false">공수1!N3</f>
@@ -26806,7 +26812,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C17" s="43" t="str">
         <f aca="false">공수1!O4</f>
@@ -26818,7 +26824,7 @@
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">공수1!O3</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F17" s="44" t="n">
         <f aca="false">IF(공수1!$O$2="","",공수1!$O$2)</f>
@@ -26882,7 +26888,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C18" s="43" t="str">
         <f aca="false">공수1!P4</f>
@@ -26894,7 +26900,7 @@
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">공수1!P3</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F18" s="44" t="n">
         <f aca="false">IF(공수1!$P$2="","",공수1!$P$2)</f>
@@ -26958,7 +26964,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C19" s="43" t="str">
         <f aca="false">공수1!Q4</f>
@@ -26970,7 +26976,7 @@
       </c>
       <c r="E19" s="10" t="n">
         <f aca="false">공수1!Q3</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="44" t="n">
         <f aca="false">IF(공수1!$Q$2="","",공수1!$Q$2)</f>
@@ -27034,7 +27040,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C20" s="43" t="str">
         <f aca="false">공수1!R4</f>
@@ -27085,19 +27091,19 @@
         <v/>
       </c>
       <c r="O20" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P20" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q20" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R20" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S20" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27105,7 +27111,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C21" s="43" t="str">
         <f aca="false">공수1!S4</f>
@@ -27113,11 +27119,11 @@
       </c>
       <c r="D21" s="10" t="str">
         <f aca="false">공수1!S5</f>
-        <v>하</v>
+        <v>중하</v>
       </c>
       <c r="E21" s="10" t="n">
         <f aca="false">공수1!S3</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F21" s="44" t="n">
         <f aca="false">IF(공수1!$S$2="","",공수1!$S$2)</f>
@@ -27156,19 +27162,19 @@
         <v/>
       </c>
       <c r="O21" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P21" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q21" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R21" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S21" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27176,7 +27182,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C22" s="43" t="str">
         <f aca="false">공수1!T4</f>
@@ -27227,19 +27233,19 @@
         <v/>
       </c>
       <c r="O22" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P22" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q22" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R22" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S22" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27247,7 +27253,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C23" s="43" t="str">
         <f aca="false">공수1!U4</f>
@@ -27298,19 +27304,19 @@
         <v/>
       </c>
       <c r="O23" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P23" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q23" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R23" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S23" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27318,7 +27324,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C24" s="43" t="str">
         <f aca="false">공수1!V4</f>
@@ -27326,7 +27332,7 @@
       </c>
       <c r="D24" s="10" t="str">
         <f aca="false">공수1!V5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E24" s="10" t="n">
         <f aca="false">공수1!V3</f>
@@ -27369,19 +27375,19 @@
         <v/>
       </c>
       <c r="O24" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P24" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q24" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R24" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S24" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27389,7 +27395,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C25" s="43" t="str">
         <f aca="false">공수1!W4</f>
@@ -27440,24 +27446,24 @@
         <v/>
       </c>
       <c r="O25" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P25" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q25" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R25" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S25" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="42" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B28" s="42"/>
       <c r="C28" s="42"/>
@@ -27466,31 +27472,31 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>25</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J29" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -27505,25 +27511,25 @@
         <v>기본반 정답률</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O29" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P29" s="19" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="Q29" s="19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R29" s="19" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S29" s="19" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27531,7 +27537,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C30" s="43" t="str">
         <f aca="false">공수2!D4</f>
@@ -27607,7 +27613,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C31" s="43" t="str">
         <f aca="false">공수2!E4</f>
@@ -27683,7 +27689,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C32" s="43" t="str">
         <f aca="false">공수2!F4</f>
@@ -27759,7 +27765,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C33" s="43" t="str">
         <f aca="false">공수2!G4</f>
@@ -27767,11 +27773,11 @@
       </c>
       <c r="D33" s="10" t="str">
         <f aca="false">공수2!G5</f>
-        <v>하</v>
+        <v>중하</v>
       </c>
       <c r="E33" s="10" t="n">
         <f aca="false">공수2!G3</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F33" s="44" t="n">
         <f aca="false">IF(공수2!$G$2="","",공수2!$G$2)</f>
@@ -27835,7 +27841,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C34" s="43" t="str">
         <f aca="false">공수2!H4</f>
@@ -27843,11 +27849,11 @@
       </c>
       <c r="D34" s="10" t="str">
         <f aca="false">공수2!H5</f>
-        <v>중</v>
+        <v>중하</v>
       </c>
       <c r="E34" s="10" t="n">
         <f aca="false">공수2!H3</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" s="44" t="n">
         <f aca="false">IF(공수2!$H$2="","",공수2!$H$2)</f>
@@ -27911,7 +27917,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C35" s="43" t="str">
         <f aca="false">공수2!I4</f>
@@ -27919,11 +27925,11 @@
       </c>
       <c r="D35" s="10" t="str">
         <f aca="false">공수2!I5</f>
-        <v>중</v>
+        <v>중하</v>
       </c>
       <c r="E35" s="10" t="n">
         <f aca="false">공수2!I3</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" s="44" t="n">
         <f aca="false">IF(공수2!$I$2="","",공수2!$I$2)</f>
@@ -27987,7 +27993,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C36" s="43" t="str">
         <f aca="false">공수2!J4</f>
@@ -28063,7 +28069,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C37" s="43" t="str">
         <f aca="false">공수2!K4</f>
@@ -28139,7 +28145,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C38" s="43" t="str">
         <f aca="false">공수2!L4</f>
@@ -28147,11 +28153,11 @@
       </c>
       <c r="D38" s="10" t="str">
         <f aca="false">공수2!L5</f>
-        <v>상</v>
+        <v>중</v>
       </c>
       <c r="E38" s="10" t="n">
         <f aca="false">공수2!L3</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" s="44" t="n">
         <f aca="false">IF(공수2!$L$2="","",공수2!$L$2)</f>
@@ -28215,7 +28221,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C39" s="43" t="str">
         <f aca="false">공수2!M4</f>
@@ -28223,7 +28229,7 @@
       </c>
       <c r="D39" s="10" t="str">
         <f aca="false">공수2!M5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E39" s="10" t="n">
         <f aca="false">공수2!M3</f>
@@ -28291,7 +28297,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C40" s="43" t="str">
         <f aca="false">공수2!N4</f>
@@ -28299,7 +28305,7 @@
       </c>
       <c r="D40" s="10" t="str">
         <f aca="false">공수2!N5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E40" s="10" t="n">
         <f aca="false">공수2!N3</f>
@@ -28367,7 +28373,7 @@
         <v>12</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C41" s="43" t="str">
         <f aca="false">공수2!O4</f>
@@ -28379,7 +28385,7 @@
       </c>
       <c r="E41" s="10" t="n">
         <f aca="false">공수2!O3</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F41" s="44" t="n">
         <f aca="false">IF(공수2!$O$2="","",공수2!$O$2)</f>
@@ -28443,7 +28449,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C42" s="43" t="str">
         <f aca="false">공수2!P4</f>
@@ -28455,7 +28461,7 @@
       </c>
       <c r="E42" s="10" t="n">
         <f aca="false">공수2!P3</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F42" s="44" t="n">
         <f aca="false">IF(공수2!$P$2="","",공수2!$P$2)</f>
@@ -28519,7 +28525,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C43" s="43" t="str">
         <f aca="false">공수2!Q4</f>
@@ -28531,7 +28537,7 @@
       </c>
       <c r="E43" s="10" t="n">
         <f aca="false">공수2!Q3</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" s="44" t="n">
         <f aca="false">IF(공수2!$Q$2="","",공수2!$Q$2)</f>
@@ -28595,7 +28601,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C44" s="43" t="str">
         <f aca="false">공수2!R4</f>
@@ -28646,19 +28652,19 @@
         <v/>
       </c>
       <c r="O44" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P44" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q44" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R44" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S44" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28666,7 +28672,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C45" s="43" t="str">
         <f aca="false">공수2!S4</f>
@@ -28674,11 +28680,11 @@
       </c>
       <c r="D45" s="10" t="str">
         <f aca="false">공수2!S5</f>
-        <v>하</v>
+        <v>중하</v>
       </c>
       <c r="E45" s="10" t="n">
         <f aca="false">공수2!S3</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F45" s="44" t="n">
         <f aca="false">IF(공수2!$S$2="","",공수2!$S$2)</f>
@@ -28717,19 +28723,19 @@
         <v/>
       </c>
       <c r="O45" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P45" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q45" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R45" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S45" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28737,7 +28743,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C46" s="43" t="str">
         <f aca="false">공수2!T4</f>
@@ -28788,19 +28794,19 @@
         <v/>
       </c>
       <c r="O46" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P46" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q46" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R46" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S46" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28808,7 +28814,7 @@
         <v>18</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C47" s="43" t="str">
         <f aca="false">공수2!U4</f>
@@ -28859,19 +28865,19 @@
         <v/>
       </c>
       <c r="O47" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P47" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q47" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R47" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S47" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28879,7 +28885,7 @@
         <v>19</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C48" s="43" t="str">
         <f aca="false">공수2!V4</f>
@@ -28887,7 +28893,7 @@
       </c>
       <c r="D48" s="10" t="str">
         <f aca="false">공수2!V5</f>
-        <v>상</v>
+        <v>중상</v>
       </c>
       <c r="E48" s="10" t="n">
         <f aca="false">공수2!V3</f>
@@ -28930,19 +28936,19 @@
         <v/>
       </c>
       <c r="O48" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P48" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q48" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R48" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S48" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28950,7 +28956,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C49" s="43" t="str">
         <f aca="false">공수2!W4</f>
@@ -29001,19 +29007,19 @@
         <v/>
       </c>
       <c r="O49" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P49" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Q49" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R49" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="S49" s="49" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fill parent report recommended class from final class in workbook
학부모 보고서 추천 반을 반배정 시트의 최종반(수동조정 우선)과 설정의
반 소개 문구로 채움. 보류·미정이면 빈칸으로 두고 생성 시 해당 학생 목록 안내.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="179">
   <si>
     <r>
       <rPr>
@@ -2799,6 +2799,287 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">무리함수의 그래프를 직접 그려 보는 학습이 필요합니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">⑥ 반 소개 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">학부모 보고서의 추천 반 아래 문구</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">소개 문구</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1·2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모두 탄탄한 기초를 갖춘 학생을 위한 반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개념 심화와 고난도 문항 해결력</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내신 상위권 대비까지 진행합니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 강점을 살리면서 공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 개념을 처음부터 체계적으로 다져</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">두 과목의 균형을 맞추는 반입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중등 연계 개념부터 차근차근 점검하며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1·2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 핵심 개념과 기본 유형을 확실히 완성하는 반입니다</t>
     </r>
     <r>
       <rPr>
@@ -4103,6 +4384,25 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최종반이 학부모 보고서의 추천 반으로 들어갑니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
     </r>
     <r>
       <rPr>
@@ -5700,7 +6000,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -6304,8 +6604,60 @@
       <c r="D51" s="20"/>
       <c r="E51" s="20"/>
     </row>
+    <row r="53" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="str">
+        <f aca="false">B6</f>
+        <v>TF1반</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+    </row>
+    <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="str">
+        <f aca="false">B7</f>
+        <v>TF2반</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+    </row>
+    <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="str">
+        <f aca="false">B8</f>
+        <v>TF3반</v>
+      </c>
+      <c r="B57" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="26">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="H5:L9"/>
@@ -6328,6 +6680,10 @@
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B57:E57"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B35" type="list">
@@ -6362,7 +6718,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6372,7 +6728,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6382,22 +6738,22 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,19 +6761,19 @@
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7250,12 +7606,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -7285,7 +7641,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -7352,7 +7708,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -7443,7 +7799,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -7510,164 +7866,164 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="Q5" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="R5" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="R5" s="14" t="s">
-        <v>100</v>
-      </c>
       <c r="S5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B19</f>
@@ -12312,12 +12668,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -12346,7 +12702,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -12413,7 +12769,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -12500,7 +12856,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -12567,161 +12923,161 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="Q5" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="R5" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="R5" s="14" t="s">
-        <v>100</v>
-      </c>
       <c r="S5" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B24</f>
@@ -17048,7 +17404,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17075,7 +17431,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -17102,69 +17458,69 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O5" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17684,7 +18040,7 @@
         <v/>
       </c>
       <c r="O13" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="P13" s="5"/>
       <c r="Q13" s="5"/>
@@ -21738,7 +22094,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -21752,7 +22108,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -21766,34 +22122,34 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25848,7 +26204,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -25870,7 +26226,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -25892,7 +26248,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="45" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B4" s="45"/>
       <c r="C4" s="45"/>
@@ -25901,31 +26257,31 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -25940,25 +26296,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="P5" s="24" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="Q5" s="24" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="R5" s="24" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="S5" s="24" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25966,7 +26322,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C6" s="46" t="str">
         <f aca="false">공수1!D4</f>
@@ -26042,7 +26398,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C7" s="46" t="str">
         <f aca="false">공수1!E4</f>
@@ -26118,7 +26474,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C8" s="46" t="str">
         <f aca="false">공수1!F4</f>
@@ -26194,7 +26550,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C9" s="46" t="str">
         <f aca="false">공수1!G4</f>
@@ -26270,7 +26626,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C10" s="46" t="str">
         <f aca="false">공수1!H4</f>
@@ -26346,7 +26702,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C11" s="46" t="str">
         <f aca="false">공수1!I4</f>
@@ -26422,7 +26778,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C12" s="46" t="str">
         <f aca="false">공수1!J4</f>
@@ -26498,7 +26854,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C13" s="46" t="str">
         <f aca="false">공수1!K4</f>
@@ -26574,7 +26930,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C14" s="46" t="str">
         <f aca="false">공수1!L4</f>
@@ -26650,7 +27006,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C15" s="46" t="str">
         <f aca="false">공수1!M4</f>
@@ -26726,7 +27082,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C16" s="46" t="str">
         <f aca="false">공수1!N4</f>
@@ -26802,7 +27158,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C17" s="46" t="str">
         <f aca="false">공수1!O4</f>
@@ -26878,7 +27234,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C18" s="46" t="str">
         <f aca="false">공수1!P4</f>
@@ -26954,7 +27310,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C19" s="46" t="str">
         <f aca="false">공수1!Q4</f>
@@ -27030,7 +27386,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C20" s="46" t="str">
         <f aca="false">공수1!R4</f>
@@ -27081,19 +27437,19 @@
         <v/>
       </c>
       <c r="O20" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P20" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q20" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R20" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S20" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27101,7 +27457,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C21" s="46" t="str">
         <f aca="false">공수1!S4</f>
@@ -27152,19 +27508,19 @@
         <v/>
       </c>
       <c r="O21" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P21" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q21" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R21" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S21" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27172,7 +27528,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C22" s="46" t="str">
         <f aca="false">공수1!T4</f>
@@ -27223,19 +27579,19 @@
         <v/>
       </c>
       <c r="O22" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P22" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q22" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R22" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S22" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27243,7 +27599,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C23" s="46" t="str">
         <f aca="false">공수1!U4</f>
@@ -27294,19 +27650,19 @@
         <v/>
       </c>
       <c r="O23" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P23" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q23" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R23" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S23" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27314,7 +27670,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C24" s="46" t="str">
         <f aca="false">공수1!V4</f>
@@ -27365,19 +27721,19 @@
         <v/>
       </c>
       <c r="O24" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P24" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q24" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R24" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S24" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27385,7 +27741,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C25" s="46" t="str">
         <f aca="false">공수1!W4</f>
@@ -27436,24 +27792,24 @@
         <v/>
       </c>
       <c r="O25" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P25" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q25" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R25" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S25" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="45" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B28" s="45"/>
       <c r="C28" s="45"/>
@@ -27462,31 +27818,31 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="J29" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -27501,25 +27857,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="O29" s="24" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="P29" s="24" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="Q29" s="24" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="R29" s="24" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="S29" s="24" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27527,7 +27883,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C30" s="46" t="str">
         <f aca="false">공수2!D4</f>
@@ -27603,7 +27959,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C31" s="46" t="str">
         <f aca="false">공수2!E4</f>
@@ -27679,7 +28035,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C32" s="46" t="str">
         <f aca="false">공수2!F4</f>
@@ -27755,7 +28111,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C33" s="46" t="str">
         <f aca="false">공수2!G4</f>
@@ -27831,7 +28187,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C34" s="46" t="str">
         <f aca="false">공수2!H4</f>
@@ -27907,7 +28263,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C35" s="46" t="str">
         <f aca="false">공수2!I4</f>
@@ -27983,7 +28339,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C36" s="46" t="str">
         <f aca="false">공수2!J4</f>
@@ -28059,7 +28415,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C37" s="46" t="str">
         <f aca="false">공수2!K4</f>
@@ -28135,7 +28491,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C38" s="46" t="str">
         <f aca="false">공수2!L4</f>
@@ -28211,7 +28567,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C39" s="46" t="str">
         <f aca="false">공수2!M4</f>
@@ -28287,7 +28643,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C40" s="46" t="str">
         <f aca="false">공수2!N4</f>
@@ -28363,7 +28719,7 @@
         <v>12</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C41" s="46" t="str">
         <f aca="false">공수2!O4</f>
@@ -28439,7 +28795,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C42" s="46" t="str">
         <f aca="false">공수2!P4</f>
@@ -28515,7 +28871,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C43" s="46" t="str">
         <f aca="false">공수2!Q4</f>
@@ -28591,7 +28947,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C44" s="46" t="str">
         <f aca="false">공수2!R4</f>
@@ -28642,19 +28998,19 @@
         <v/>
       </c>
       <c r="O44" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P44" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q44" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R44" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S44" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28662,7 +29018,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C45" s="46" t="str">
         <f aca="false">공수2!S4</f>
@@ -28713,19 +29069,19 @@
         <v/>
       </c>
       <c r="O45" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P45" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q45" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R45" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S45" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28733,7 +29089,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C46" s="46" t="str">
         <f aca="false">공수2!T4</f>
@@ -28784,19 +29140,19 @@
         <v/>
       </c>
       <c r="O46" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P46" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q46" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R46" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S46" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28804,7 +29160,7 @@
         <v>18</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C47" s="46" t="str">
         <f aca="false">공수2!U4</f>
@@ -28855,19 +29211,19 @@
         <v/>
       </c>
       <c r="O47" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P47" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q47" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R47" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S47" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28875,7 +29231,7 @@
         <v>19</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C48" s="46" t="str">
         <f aca="false">공수2!V4</f>
@@ -28926,19 +29282,19 @@
         <v/>
       </c>
       <c r="O48" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P48" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q48" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R48" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S48" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28946,7 +29302,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C49" s="46" t="str">
         <f aca="false">공수2!W4</f>
@@ -28997,19 +29353,19 @@
         <v/>
       </c>
       <c r="O49" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P49" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q49" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="R49" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="S49" s="52" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add previous class and learning progress columns to student list
학생명단에 기존 반명(신규 학생은 '신규')과 학습 진도 열을 추가하고
상담 카드 상단에 함께 표시.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="183">
   <si>
     <r>
       <rPr>
@@ -3227,7 +3227,83 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">.</t>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기존 반명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재원생은 현재 반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신규 학생은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신규</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'.</t>
     </r>
   </si>
   <si>
@@ -3243,6 +3319,12 @@
     <t xml:space="preserve">구분</t>
   </si>
   <si>
+    <t xml:space="preserve">기존 반명</t>
+  </si>
+  <si>
+    <t xml:space="preserve">학습 진도</t>
+  </si>
+  <si>
     <t xml:space="preserve">연락처</t>
   </si>
   <si>
@@ -3352,6 +3434,77 @@
   </si>
   <si>
     <t xml:space="preserve">외부</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신규</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회독 완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">집합까지</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">010-0000-0000</t>
@@ -6706,14 +6859,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6725,6 +6880,8 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -6735,6 +6892,8 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
@@ -6755,25 +6914,37 @@
       <c r="F6" s="4" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>99</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>98</v>
+        <v>100</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="H7" s="25" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6785,6 +6956,8 @@
       <c r="D8" s="14"/>
       <c r="E8" s="8"/>
       <c r="F8" s="25"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
@@ -6795,6 +6968,8 @@
       <c r="D9" s="14"/>
       <c r="E9" s="8"/>
       <c r="F9" s="25"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
@@ -6805,6 +6980,8 @@
       <c r="D10" s="14"/>
       <c r="E10" s="8"/>
       <c r="F10" s="25"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
@@ -6815,6 +6992,8 @@
       <c r="D11" s="14"/>
       <c r="E11" s="8"/>
       <c r="F11" s="25"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
@@ -6825,6 +7004,8 @@
       <c r="D12" s="14"/>
       <c r="E12" s="8"/>
       <c r="F12" s="25"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
@@ -6835,6 +7016,8 @@
       <c r="D13" s="14"/>
       <c r="E13" s="8"/>
       <c r="F13" s="25"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
@@ -6845,6 +7028,8 @@
       <c r="D14" s="14"/>
       <c r="E14" s="8"/>
       <c r="F14" s="25"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="n">
@@ -6855,6 +7040,8 @@
       <c r="D15" s="14"/>
       <c r="E15" s="8"/>
       <c r="F15" s="25"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="25"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
@@ -6865,6 +7052,8 @@
       <c r="D16" s="14"/>
       <c r="E16" s="8"/>
       <c r="F16" s="25"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="25"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="n">
@@ -6875,6 +7064,8 @@
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
       <c r="F17" s="25"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
@@ -6885,6 +7076,8 @@
       <c r="D18" s="14"/>
       <c r="E18" s="8"/>
       <c r="F18" s="25"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="25"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="n">
@@ -6895,6 +7088,8 @@
       <c r="D19" s="14"/>
       <c r="E19" s="8"/>
       <c r="F19" s="25"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="25"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
@@ -6905,6 +7100,8 @@
       <c r="D20" s="14"/>
       <c r="E20" s="8"/>
       <c r="F20" s="25"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="25"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="n">
@@ -6915,6 +7112,8 @@
       <c r="D21" s="14"/>
       <c r="E21" s="8"/>
       <c r="F21" s="25"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="25"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="n">
@@ -6925,6 +7124,8 @@
       <c r="D22" s="14"/>
       <c r="E22" s="8"/>
       <c r="F22" s="25"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="25"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="n">
@@ -6935,6 +7136,8 @@
       <c r="D23" s="14"/>
       <c r="E23" s="8"/>
       <c r="F23" s="25"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="25"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="n">
@@ -6945,6 +7148,8 @@
       <c r="D24" s="14"/>
       <c r="E24" s="8"/>
       <c r="F24" s="25"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="25"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="n">
@@ -6955,6 +7160,8 @@
       <c r="D25" s="14"/>
       <c r="E25" s="8"/>
       <c r="F25" s="25"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="25"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="n">
@@ -6965,6 +7172,8 @@
       <c r="D26" s="14"/>
       <c r="E26" s="8"/>
       <c r="F26" s="25"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="25"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="n">
@@ -6975,6 +7184,8 @@
       <c r="D27" s="14"/>
       <c r="E27" s="8"/>
       <c r="F27" s="25"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="25"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="n">
@@ -6985,6 +7196,8 @@
       <c r="D28" s="14"/>
       <c r="E28" s="8"/>
       <c r="F28" s="25"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="25"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="n">
@@ -6995,6 +7208,8 @@
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
       <c r="F29" s="25"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="25"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="n">
@@ -7005,6 +7220,8 @@
       <c r="D30" s="14"/>
       <c r="E30" s="8"/>
       <c r="F30" s="25"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="25"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="n">
@@ -7015,6 +7232,8 @@
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
       <c r="F31" s="25"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="25"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="n">
@@ -7025,6 +7244,8 @@
       <c r="D32" s="14"/>
       <c r="E32" s="8"/>
       <c r="F32" s="25"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="25"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="n">
@@ -7035,6 +7256,8 @@
       <c r="D33" s="14"/>
       <c r="E33" s="8"/>
       <c r="F33" s="25"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="25"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="n">
@@ -7045,6 +7268,8 @@
       <c r="D34" s="14"/>
       <c r="E34" s="8"/>
       <c r="F34" s="25"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="25"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="n">
@@ -7055,6 +7280,8 @@
       <c r="D35" s="14"/>
       <c r="E35" s="8"/>
       <c r="F35" s="25"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="25"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="n">
@@ -7065,6 +7292,8 @@
       <c r="D36" s="14"/>
       <c r="E36" s="8"/>
       <c r="F36" s="25"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="25"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="n">
@@ -7075,6 +7304,8 @@
       <c r="D37" s="14"/>
       <c r="E37" s="8"/>
       <c r="F37" s="25"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="25"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="n">
@@ -7085,6 +7316,8 @@
       <c r="D38" s="14"/>
       <c r="E38" s="8"/>
       <c r="F38" s="25"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="25"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="n">
@@ -7095,6 +7328,8 @@
       <c r="D39" s="14"/>
       <c r="E39" s="8"/>
       <c r="F39" s="25"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="25"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="n">
@@ -7105,6 +7340,8 @@
       <c r="D40" s="14"/>
       <c r="E40" s="8"/>
       <c r="F40" s="25"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="25"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="n">
@@ -7115,6 +7352,8 @@
       <c r="D41" s="14"/>
       <c r="E41" s="8"/>
       <c r="F41" s="25"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="25"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="n">
@@ -7125,6 +7364,8 @@
       <c r="D42" s="14"/>
       <c r="E42" s="8"/>
       <c r="F42" s="25"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="25"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="n">
@@ -7135,6 +7376,8 @@
       <c r="D43" s="14"/>
       <c r="E43" s="8"/>
       <c r="F43" s="25"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="25"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="n">
@@ -7145,6 +7388,8 @@
       <c r="D44" s="14"/>
       <c r="E44" s="8"/>
       <c r="F44" s="25"/>
+      <c r="G44" s="8"/>
+      <c r="H44" s="25"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="n">
@@ -7155,6 +7400,8 @@
       <c r="D45" s="14"/>
       <c r="E45" s="8"/>
       <c r="F45" s="25"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="25"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="n">
@@ -7165,6 +7412,8 @@
       <c r="D46" s="14"/>
       <c r="E46" s="8"/>
       <c r="F46" s="25"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="25"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="n">
@@ -7175,6 +7424,8 @@
       <c r="D47" s="14"/>
       <c r="E47" s="8"/>
       <c r="F47" s="25"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="25"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="n">
@@ -7185,6 +7436,8 @@
       <c r="D48" s="14"/>
       <c r="E48" s="8"/>
       <c r="F48" s="25"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="25"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="n">
@@ -7195,6 +7448,8 @@
       <c r="D49" s="14"/>
       <c r="E49" s="8"/>
       <c r="F49" s="25"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="25"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="n">
@@ -7205,6 +7460,8 @@
       <c r="D50" s="14"/>
       <c r="E50" s="8"/>
       <c r="F50" s="25"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="25"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="n">
@@ -7215,6 +7472,8 @@
       <c r="D51" s="14"/>
       <c r="E51" s="8"/>
       <c r="F51" s="25"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="25"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="n">
@@ -7225,6 +7484,8 @@
       <c r="D52" s="14"/>
       <c r="E52" s="8"/>
       <c r="F52" s="25"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="25"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="n">
@@ -7235,6 +7496,8 @@
       <c r="D53" s="14"/>
       <c r="E53" s="8"/>
       <c r="F53" s="25"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="25"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="n">
@@ -7245,6 +7508,8 @@
       <c r="D54" s="14"/>
       <c r="E54" s="8"/>
       <c r="F54" s="25"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="25"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="n">
@@ -7255,6 +7520,8 @@
       <c r="D55" s="14"/>
       <c r="E55" s="8"/>
       <c r="F55" s="25"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="25"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="n">
@@ -7265,6 +7532,8 @@
       <c r="D56" s="14"/>
       <c r="E56" s="8"/>
       <c r="F56" s="25"/>
+      <c r="G56" s="8"/>
+      <c r="H56" s="25"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="n">
@@ -7275,6 +7544,8 @@
       <c r="D57" s="14"/>
       <c r="E57" s="8"/>
       <c r="F57" s="25"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="25"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="n">
@@ -7285,6 +7556,8 @@
       <c r="D58" s="14"/>
       <c r="E58" s="8"/>
       <c r="F58" s="25"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="25"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="n">
@@ -7295,6 +7568,8 @@
       <c r="D59" s="14"/>
       <c r="E59" s="8"/>
       <c r="F59" s="25"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="25"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="n">
@@ -7305,6 +7580,8 @@
       <c r="D60" s="14"/>
       <c r="E60" s="8"/>
       <c r="F60" s="25"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="25"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="n">
@@ -7315,6 +7592,8 @@
       <c r="D61" s="14"/>
       <c r="E61" s="8"/>
       <c r="F61" s="25"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="25"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="n">
@@ -7325,6 +7604,8 @@
       <c r="D62" s="14"/>
       <c r="E62" s="8"/>
       <c r="F62" s="25"/>
+      <c r="G62" s="8"/>
+      <c r="H62" s="25"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="n">
@@ -7335,6 +7616,8 @@
       <c r="D63" s="14"/>
       <c r="E63" s="8"/>
       <c r="F63" s="25"/>
+      <c r="G63" s="8"/>
+      <c r="H63" s="25"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="n">
@@ -7345,6 +7628,8 @@
       <c r="D64" s="14"/>
       <c r="E64" s="8"/>
       <c r="F64" s="25"/>
+      <c r="G64" s="8"/>
+      <c r="H64" s="25"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="n">
@@ -7355,6 +7640,8 @@
       <c r="D65" s="14"/>
       <c r="E65" s="8"/>
       <c r="F65" s="25"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="25"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="n">
@@ -7365,6 +7652,8 @@
       <c r="D66" s="14"/>
       <c r="E66" s="8"/>
       <c r="F66" s="25"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="25"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="n">
@@ -7375,6 +7664,8 @@
       <c r="D67" s="14"/>
       <c r="E67" s="8"/>
       <c r="F67" s="25"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="25"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="n">
@@ -7385,6 +7676,8 @@
       <c r="D68" s="14"/>
       <c r="E68" s="8"/>
       <c r="F68" s="25"/>
+      <c r="G68" s="8"/>
+      <c r="H68" s="25"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="n">
@@ -7395,6 +7688,8 @@
       <c r="D69" s="14"/>
       <c r="E69" s="8"/>
       <c r="F69" s="25"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="25"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="n">
@@ -7405,6 +7700,8 @@
       <c r="D70" s="14"/>
       <c r="E70" s="8"/>
       <c r="F70" s="25"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="25"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="n">
@@ -7415,6 +7712,8 @@
       <c r="D71" s="14"/>
       <c r="E71" s="8"/>
       <c r="F71" s="25"/>
+      <c r="G71" s="8"/>
+      <c r="H71" s="25"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="n">
@@ -7425,6 +7724,8 @@
       <c r="D72" s="14"/>
       <c r="E72" s="8"/>
       <c r="F72" s="25"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="25"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="n">
@@ -7435,6 +7736,8 @@
       <c r="D73" s="14"/>
       <c r="E73" s="8"/>
       <c r="F73" s="25"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="25"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="n">
@@ -7445,6 +7748,8 @@
       <c r="D74" s="14"/>
       <c r="E74" s="8"/>
       <c r="F74" s="25"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="25"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="n">
@@ -7455,6 +7760,8 @@
       <c r="D75" s="14"/>
       <c r="E75" s="8"/>
       <c r="F75" s="25"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="25"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="n">
@@ -7465,6 +7772,8 @@
       <c r="D76" s="14"/>
       <c r="E76" s="8"/>
       <c r="F76" s="25"/>
+      <c r="G76" s="8"/>
+      <c r="H76" s="25"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="n">
@@ -7475,6 +7784,8 @@
       <c r="D77" s="14"/>
       <c r="E77" s="8"/>
       <c r="F77" s="25"/>
+      <c r="G77" s="8"/>
+      <c r="H77" s="25"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="n">
@@ -7485,6 +7796,8 @@
       <c r="D78" s="14"/>
       <c r="E78" s="8"/>
       <c r="F78" s="25"/>
+      <c r="G78" s="8"/>
+      <c r="H78" s="25"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="n">
@@ -7495,6 +7808,8 @@
       <c r="D79" s="14"/>
       <c r="E79" s="8"/>
       <c r="F79" s="25"/>
+      <c r="G79" s="8"/>
+      <c r="H79" s="25"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="n">
@@ -7505,6 +7820,8 @@
       <c r="D80" s="14"/>
       <c r="E80" s="8"/>
       <c r="F80" s="25"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="25"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="n">
@@ -7515,6 +7832,8 @@
       <c r="D81" s="14"/>
       <c r="E81" s="8"/>
       <c r="F81" s="25"/>
+      <c r="G81" s="8"/>
+      <c r="H81" s="25"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="n">
@@ -7525,6 +7844,8 @@
       <c r="D82" s="14"/>
       <c r="E82" s="8"/>
       <c r="F82" s="25"/>
+      <c r="G82" s="8"/>
+      <c r="H82" s="25"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="n">
@@ -7535,6 +7856,8 @@
       <c r="D83" s="14"/>
       <c r="E83" s="8"/>
       <c r="F83" s="25"/>
+      <c r="G83" s="8"/>
+      <c r="H83" s="25"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="n">
@@ -7545,6 +7868,8 @@
       <c r="D84" s="14"/>
       <c r="E84" s="8"/>
       <c r="F84" s="25"/>
+      <c r="G84" s="8"/>
+      <c r="H84" s="25"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="n">
@@ -7555,6 +7880,8 @@
       <c r="D85" s="14"/>
       <c r="E85" s="8"/>
       <c r="F85" s="25"/>
+      <c r="G85" s="8"/>
+      <c r="H85" s="25"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="n">
@@ -7565,11 +7892,13 @@
       <c r="D86" s="14"/>
       <c r="E86" s="8"/>
       <c r="F86" s="25"/>
+      <c r="G86" s="8"/>
+      <c r="H86" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D7:D86" type="list">
@@ -7606,12 +7935,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -7641,7 +7970,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -7708,7 +8037,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -7799,7 +8128,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -7866,87 +8195,87 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="O5" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="R5" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="P5" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q5" s="14" t="s">
+      <c r="S5" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="R5" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="S5" s="14" t="s">
-        <v>106</v>
-      </c>
       <c r="T5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7960,70 +8289,70 @@
         <v>90</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B19</f>
@@ -12622,6 +12951,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
+      <formula1>설정!$B$19:$B$22</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
+      <formula1>"하,중하,중,중상,상,최상"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -12629,14 +12966,6 @@
     <dataValidation allowBlank="true" error="단답형은 0~999 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R2:W2 R7:W86" type="whole">
       <formula1>0</formula1>
       <formula2>999</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
-      <formula1>설정!$B$19:$B$22</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
-      <formula1>"하,중하,중,중상,상,최상"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12668,12 +12997,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -12702,7 +13031,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -12769,7 +13098,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -12856,7 +13185,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -12923,84 +13252,84 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="O5" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="R5" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="P5" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q5" s="14" t="s">
+      <c r="S5" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="R5" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="S5" s="14" t="s">
-        <v>106</v>
-      </c>
       <c r="T5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13014,70 +13343,70 @@
         <v>90</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B24</f>
@@ -17352,6 +17681,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="단답형은 0~999 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R2:W2 R7:W86" type="whole">
+      <formula1>0</formula1>
+      <formula2>999</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
       <formula1>설정!$B$24:$B$26</formula1>
       <formula2>0</formula2>
@@ -17359,14 +17696,6 @@
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
       <formula1>"하,중하,중,중상,상,최상"</formula1>
       <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
-      <formula1>1</formula1>
-      <formula2>5</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="단답형은 0~999 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R2:W2 R7:W86" type="whole">
-      <formula1>0</formula1>
-      <formula2>999</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -17404,7 +17733,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17431,7 +17760,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -17458,7 +17787,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O5" s="3" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17475,52 +17804,52 @@
         <v>91</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18040,7 +18369,7 @@
         <v/>
       </c>
       <c r="O13" s="5" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="P13" s="5"/>
       <c r="Q13" s="5"/>
@@ -22094,7 +22423,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -22108,7 +22437,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -22122,7 +22451,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>89</v>
@@ -22134,22 +22463,22 @@
         <v>91</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26204,7 +26533,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -26226,7 +26555,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -26248,7 +26577,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="45" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B4" s="45"/>
       <c r="C4" s="45"/>
@@ -26257,31 +26586,31 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -26296,25 +26625,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="P5" s="24" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="Q5" s="24" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="R5" s="24" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="S5" s="24" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26322,7 +26651,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C6" s="46" t="str">
         <f aca="false">공수1!D4</f>
@@ -26398,7 +26727,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C7" s="46" t="str">
         <f aca="false">공수1!E4</f>
@@ -26474,7 +26803,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C8" s="46" t="str">
         <f aca="false">공수1!F4</f>
@@ -26550,7 +26879,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C9" s="46" t="str">
         <f aca="false">공수1!G4</f>
@@ -26626,7 +26955,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C10" s="46" t="str">
         <f aca="false">공수1!H4</f>
@@ -26702,7 +27031,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C11" s="46" t="str">
         <f aca="false">공수1!I4</f>
@@ -26778,7 +27107,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C12" s="46" t="str">
         <f aca="false">공수1!J4</f>
@@ -26854,7 +27183,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C13" s="46" t="str">
         <f aca="false">공수1!K4</f>
@@ -26930,7 +27259,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C14" s="46" t="str">
         <f aca="false">공수1!L4</f>
@@ -27006,7 +27335,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C15" s="46" t="str">
         <f aca="false">공수1!M4</f>
@@ -27082,7 +27411,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C16" s="46" t="str">
         <f aca="false">공수1!N4</f>
@@ -27158,7 +27487,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C17" s="46" t="str">
         <f aca="false">공수1!O4</f>
@@ -27234,7 +27563,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C18" s="46" t="str">
         <f aca="false">공수1!P4</f>
@@ -27310,7 +27639,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C19" s="46" t="str">
         <f aca="false">공수1!Q4</f>
@@ -27386,7 +27715,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C20" s="46" t="str">
         <f aca="false">공수1!R4</f>
@@ -27437,19 +27766,19 @@
         <v/>
       </c>
       <c r="O20" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P20" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q20" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R20" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S20" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27457,7 +27786,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C21" s="46" t="str">
         <f aca="false">공수1!S4</f>
@@ -27508,19 +27837,19 @@
         <v/>
       </c>
       <c r="O21" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P21" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q21" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R21" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S21" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27528,7 +27857,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C22" s="46" t="str">
         <f aca="false">공수1!T4</f>
@@ -27579,19 +27908,19 @@
         <v/>
       </c>
       <c r="O22" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P22" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q22" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R22" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S22" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27599,7 +27928,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C23" s="46" t="str">
         <f aca="false">공수1!U4</f>
@@ -27650,19 +27979,19 @@
         <v/>
       </c>
       <c r="O23" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P23" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q23" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R23" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S23" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27670,7 +27999,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C24" s="46" t="str">
         <f aca="false">공수1!V4</f>
@@ -27721,19 +28050,19 @@
         <v/>
       </c>
       <c r="O24" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P24" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q24" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R24" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S24" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27741,7 +28070,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C25" s="46" t="str">
         <f aca="false">공수1!W4</f>
@@ -27792,24 +28121,24 @@
         <v/>
       </c>
       <c r="O25" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P25" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q25" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R25" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S25" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="45" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B28" s="45"/>
       <c r="C28" s="45"/>
@@ -27818,31 +28147,31 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J29" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -27857,25 +28186,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="O29" s="24" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="P29" s="24" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="Q29" s="24" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="R29" s="24" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="S29" s="24" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27883,7 +28212,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C30" s="46" t="str">
         <f aca="false">공수2!D4</f>
@@ -27959,7 +28288,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C31" s="46" t="str">
         <f aca="false">공수2!E4</f>
@@ -28035,7 +28364,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C32" s="46" t="str">
         <f aca="false">공수2!F4</f>
@@ -28111,7 +28440,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C33" s="46" t="str">
         <f aca="false">공수2!G4</f>
@@ -28187,7 +28516,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C34" s="46" t="str">
         <f aca="false">공수2!H4</f>
@@ -28263,7 +28592,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C35" s="46" t="str">
         <f aca="false">공수2!I4</f>
@@ -28339,7 +28668,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C36" s="46" t="str">
         <f aca="false">공수2!J4</f>
@@ -28415,7 +28744,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C37" s="46" t="str">
         <f aca="false">공수2!K4</f>
@@ -28491,7 +28820,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C38" s="46" t="str">
         <f aca="false">공수2!L4</f>
@@ -28567,7 +28896,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C39" s="46" t="str">
         <f aca="false">공수2!M4</f>
@@ -28643,7 +28972,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C40" s="46" t="str">
         <f aca="false">공수2!N4</f>
@@ -28719,7 +29048,7 @@
         <v>12</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C41" s="46" t="str">
         <f aca="false">공수2!O4</f>
@@ -28795,7 +29124,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C42" s="46" t="str">
         <f aca="false">공수2!P4</f>
@@ -28871,7 +29200,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C43" s="46" t="str">
         <f aca="false">공수2!Q4</f>
@@ -28947,7 +29276,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C44" s="46" t="str">
         <f aca="false">공수2!R4</f>
@@ -28998,19 +29327,19 @@
         <v/>
       </c>
       <c r="O44" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P44" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q44" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R44" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S44" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29018,7 +29347,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C45" s="46" t="str">
         <f aca="false">공수2!S4</f>
@@ -29069,19 +29398,19 @@
         <v/>
       </c>
       <c r="O45" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P45" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q45" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R45" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S45" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29089,7 +29418,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C46" s="46" t="str">
         <f aca="false">공수2!T4</f>
@@ -29140,19 +29469,19 @@
         <v/>
       </c>
       <c r="O46" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P46" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q46" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R46" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S46" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29160,7 +29489,7 @@
         <v>18</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C47" s="46" t="str">
         <f aca="false">공수2!U4</f>
@@ -29211,19 +29540,19 @@
         <v/>
       </c>
       <c r="O47" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P47" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q47" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R47" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S47" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29231,7 +29560,7 @@
         <v>19</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C48" s="46" t="str">
         <f aca="false">공수2!V4</f>
@@ -29282,19 +29611,19 @@
         <v/>
       </c>
       <c r="O48" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P48" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q48" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R48" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S48" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29302,7 +29631,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C49" s="46" t="str">
         <f aca="false">공수2!W4</f>
@@ -29353,19 +29682,19 @@
         <v/>
       </c>
       <c r="O49" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="P49" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q49" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="R49" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="S49" s="52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure recommendations into common-math class plus advanced class, add logo
수강 구조에 맞게 추천 반을 공통수학반 1개(진단평가 결과 기준)와 선행 과목반
1개(학습 진도 기준)로 변경하고 각 카드에 추천 근거 표시. 설정 시트에 선행
과목반 목록(⑦)과 반배정 입력 칸 추가. 보고서 제목·라벨에서 '반편성'과
TEST REPORT 문구 제거, 머리말에 CLIMATH 로고 이미지 적용(PDF·한글).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="198">
   <si>
     <r>
       <rPr>
@@ -1925,7 +1925,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">반편성 진단평가 결과 보고서</t>
+      <t xml:space="preserve">진단평가 결과 보고서</t>
     </r>
   </si>
   <si>
@@ -2820,7 +2820,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">⑥ 반 소개 </t>
+      <t xml:space="preserve">⑥ 공통수학반 소개 </t>
     </r>
     <r>
       <rPr>
@@ -2841,7 +2841,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">학부모 보고서 추천 반 카드 문구 </t>
+      <t xml:space="preserve">공통수학 시험 결과로 배정 </t>
     </r>
     <r>
       <rPr>
@@ -2862,7 +2862,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 선택 목록</t>
+      <t xml:space="preserve">학부모 보고서 문구 </t>
     </r>
     <r>
       <rPr>
@@ -2873,8 +2873,32 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선택 목록</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">)</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">공통수학반 이름</t>
   </si>
   <si>
     <t xml:space="preserve">소개 문구</t>
@@ -3114,7 +3138,428 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">← 추천할 반이 더 있으면 반 이름과 소개를 추가</t>
+    <t xml:space="preserve">← 공통수학반이 더 있으면 반 이름과 소개를 추가</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">⑦ 선행 과목반 소개 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">학습 진도에 따라 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과목 선택 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">학부모 보고서 문구 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선택 목록</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">선행 과목반 이름</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대수반</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지수와 로그</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지수함수와 로그함수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">삼각함수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수열을 선행하는 반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학을 마친 학생이 다음 단계로 나아가기 좋은 과정입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">← 실제 운영하는 선행반 이름</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">소개로 수정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빈 줄에 추가 가능</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">미적분Ⅰ반</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">함수의 극한과 연속</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미분</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적분을 선행하는 반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대수 학습을 마친 학생에게 권장하는 과정입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">확률과 통계반</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">순열과 조합</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확률</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통계를 선행하는 반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학의 경우의 수를 바탕으로 개념을 넓혀 가는 과정입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">학생 명단</t>
@@ -4376,7 +4821,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">절대평가</t>
+      <t xml:space="preserve">공통수학반 </t>
     </r>
     <r>
       <rPr>
@@ -4387,6 +4832,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선행 과목반</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">)</t>
     </r>
   </si>
@@ -4398,7 +4864,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">자동배정 </t>
+      <t xml:space="preserve">학생마다 </t>
     </r>
     <r>
       <rPr>
@@ -4408,7 +4874,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= '</t>
+      <t xml:space="preserve">2</t>
     </r>
     <r>
       <rPr>
@@ -4417,7 +4883,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">설정</t>
+      <t xml:space="preserve">개 반 수강</t>
     </r>
     <r>
       <rPr>
@@ -4427,7 +4893,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">' ①</t>
+      <t xml:space="preserve">: ① </t>
     </r>
     <r>
       <rPr>
@@ -4436,7 +4902,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">의 과목별 점수 기준</t>
+      <t xml:space="preserve">공통수학반 </t>
     </r>
     <r>
       <rPr>
@@ -4446,7 +4912,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
+      <t xml:space="preserve">= </t>
     </r>
     <r>
       <rPr>
@@ -4455,7 +4921,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">해당 없으면 </t>
+      <t xml:space="preserve">시험 결과 기준 자동배정</t>
     </r>
     <r>
       <rPr>
@@ -4465,7 +4931,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">'</t>
+      <t xml:space="preserve">('</t>
     </r>
     <r>
       <rPr>
@@ -4474,7 +4940,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">보류</t>
+      <t xml:space="preserve">설정</t>
     </r>
     <r>
       <rPr>
@@ -4484,7 +4950,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">'. </t>
+      <t xml:space="preserve">' ①, </t>
     </r>
     <r>
       <rPr>
@@ -4493,7 +4959,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">노란 칸 </t>
+      <t xml:space="preserve">해당 없으면 보류</t>
     </r>
     <r>
       <rPr>
@@ -4503,7 +4969,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">'</t>
+      <t xml:space="preserve">). </t>
     </r>
     <r>
       <rPr>
@@ -4512,7 +4978,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">노란 칸 </t>
     </r>
     <r>
       <rPr>
@@ -4522,7 +4988,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1·2'</t>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -4531,7 +4997,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">에 상담 후 반을 적으면 최종반 </t>
+      <t xml:space="preserve">공통수학반</t>
     </r>
     <r>
       <rPr>
@@ -4541,7 +5007,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= </t>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -4550,7 +5016,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">에 적으면 그 반이 우선</t>
     </r>
     <r>
       <rPr>
@@ -4560,7 +5026,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1(</t>
+      <t xml:space="preserve">. ② </t>
     </r>
     <r>
       <rPr>
@@ -4569,7 +5035,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">비어 있으면 자동배정</t>
+      <t xml:space="preserve">선행반 </t>
     </r>
     <r>
       <rPr>
@@ -4579,7 +5045,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">). </t>
+      <t xml:space="preserve">= </t>
     </r>
     <r>
       <rPr>
@@ -4588,7 +5054,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">학부모 보고서에는 최종반이 </t>
+      <t xml:space="preserve">학습 진도를 보고 노란 칸 </t>
     </r>
     <r>
       <rPr>
@@ -4598,7 +5064,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1</t>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -4607,7 +5073,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">순위</t>
+      <t xml:space="preserve">선행반</t>
     </r>
     <r>
       <rPr>
@@ -4617,7 +5083,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -4626,7 +5092,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">에서 </t>
     </r>
     <r>
       <rPr>
@@ -4636,7 +5102,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
+      <t xml:space="preserve">1</t>
     </r>
     <r>
       <rPr>
@@ -4645,7 +5111,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">가 </t>
+      <t xml:space="preserve">과목 선택</t>
     </r>
     <r>
       <rPr>
@@ -4655,7 +5121,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
+      <t xml:space="preserve">('</t>
     </r>
     <r>
       <rPr>
@@ -4664,7 +5130,45 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">순위로 들어갑니다</t>
+      <t xml:space="preserve">설정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' ⑦ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">두 반 모두 학부모 보고서에 들어갑니다</t>
     </r>
     <r>
       <rPr>
@@ -4724,7 +5228,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">반별 요약 </t>
+      <t xml:space="preserve">공통수학반별 요약 </t>
     </r>
     <r>
       <rPr>
@@ -4745,7 +5249,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">최종반 기준</t>
+      <t xml:space="preserve">최종 기준</t>
     </r>
     <r>
       <rPr>
@@ -4829,7 +5333,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">공통수학반
+</t>
     </r>
     <r>
       <rPr>
@@ -4840,10 +5345,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">(</t>
+    </r>
     <r>
       <rPr>
         <b val="true"/>
@@ -4852,7 +5355,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">입력</t>
     </r>
     <r>
       <rPr>
@@ -4863,11 +5366,98 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">최종반</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선행반
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">입력</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공통수학반
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최종</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">비고</t>
@@ -5088,7 +5678,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">추천 반 </t>
+      <t xml:space="preserve">공통수학반</t>
     </r>
     <r>
       <rPr>
@@ -5098,7 +5688,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1·2</t>
+      <t xml:space="preserve">·</t>
     </r>
     <r>
       <rPr>
@@ -5107,7 +5697,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">는 목록에서 고르거나 직접 입력</t>
+      <t xml:space="preserve">선행반은 목록에서 고르거나 직접 입력</t>
     </r>
     <r>
       <rPr>
@@ -5136,7 +5726,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">' ⑥</t>
+      <t xml:space="preserve">' ⑥·⑦</t>
     </r>
     <r>
       <rPr>
@@ -5291,6 +5881,12 @@
       </rPr>
       <t xml:space="preserve">.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">공통수학반</t>
+  </si>
+  <si>
+    <t xml:space="preserve">선행반</t>
   </si>
   <si>
     <t xml:space="preserve">문항 분석</t>
@@ -6401,7 +6997,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -7005,17 +7601,17 @@
       <c r="D51" s="20"/>
       <c r="E51" s="20"/>
     </row>
-    <row r="53" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>4</v>
+        <v>82</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
@@ -7027,7 +7623,7 @@
         <v>TF1반</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C55" s="20"/>
       <c r="D55" s="20"/>
@@ -7039,7 +7635,7 @@
         <v>TF2반</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C56" s="20"/>
       <c r="D56" s="20"/>
@@ -7051,7 +7647,7 @@
         <v>TF3반</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C57" s="20"/>
       <c r="D57" s="20"/>
@@ -7064,7 +7660,7 @@
       <c r="D58" s="19"/>
       <c r="E58" s="19"/>
       <c r="F58" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7081,8 +7677,81 @@
       <c r="D60" s="19"/>
       <c r="E60" s="19"/>
     </row>
+    <row r="62" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+    </row>
+    <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B64" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+    </row>
+    <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B66" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+    </row>
+    <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7"/>
+      <c r="B67" s="19"/>
+      <c r="C67" s="19"/>
+      <c r="D67" s="19"/>
+      <c r="E67" s="19"/>
+    </row>
+    <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7"/>
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="19"/>
+    </row>
+    <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7"/>
+      <c r="B69" s="19"/>
+      <c r="C69" s="19"/>
+      <c r="D69" s="19"/>
+      <c r="E69" s="19"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="36">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="H5:L9"/>
@@ -7112,6 +7781,13 @@
     <mergeCell ref="B58:E58"/>
     <mergeCell ref="B59:E59"/>
     <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B35" type="list">
@@ -7148,7 +7824,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7160,7 +7836,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7172,28 +7848,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7201,25 +7877,25 @@
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8210,12 +8886,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -8245,7 +8921,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -8312,7 +8988,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -8403,7 +9079,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -8470,164 +9146,164 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="Q5" s="14" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="R5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="S5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B19</f>
@@ -13226,6 +13902,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
+      <formula1>"하,중하,중,중상,상,최상"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -13236,10 +13916,6 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
       <formula1>설정!$B$19:$B$22</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
-      <formula1>"하,중하,중,중상,상,최상"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -13272,12 +13948,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -13306,7 +13982,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -13373,7 +14049,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -13460,7 +14136,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -13527,161 +14203,161 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="Q5" s="14" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="R5" s="14" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="S5" s="14" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="Y5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AA5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="AB5" s="30" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="L6" s="31" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="M6" s="31" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="O6" s="31" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="P6" s="31" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="Q6" s="31" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="R6" s="32" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="S6" s="32" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="U6" s="32" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="V6" s="32" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="W6" s="32" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B24</f>
@@ -18011,7 +18687,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -18040,7 +18716,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -18067,80 +18743,80 @@
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="56.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="S5" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18723,7 +19399,7 @@
         <v/>
       </c>
       <c r="S13" s="5" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
@@ -23405,9 +24081,13 @@
       <formula>AND($O7&lt;&gt;"",$O7=설정!$B$9)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M7:N86" type="list">
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M7:M86" type="list">
       <formula1>설정!$A$55:$A$60</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N7:N86" type="list">
+      <formula1>설정!$A$64:$A$69</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -23443,7 +24123,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -23459,7 +24139,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -23475,40 +24155,40 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28203,7 +28883,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -28225,7 +28905,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -28247,7 +28927,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="46" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B4" s="46"/>
       <c r="C4" s="46"/>
@@ -28256,31 +28936,31 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -28295,25 +28975,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="P5" s="24" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="Q5" s="24" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="R5" s="24" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="S5" s="24" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28321,7 +29001,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C6" s="47" t="str">
         <f aca="false">공수1!D4</f>
@@ -28397,7 +29077,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C7" s="47" t="str">
         <f aca="false">공수1!E4</f>
@@ -28473,7 +29153,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C8" s="47" t="str">
         <f aca="false">공수1!F4</f>
@@ -28549,7 +29229,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C9" s="47" t="str">
         <f aca="false">공수1!G4</f>
@@ -28625,7 +29305,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C10" s="47" t="str">
         <f aca="false">공수1!H4</f>
@@ -28701,7 +29381,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C11" s="47" t="str">
         <f aca="false">공수1!I4</f>
@@ -28777,7 +29457,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C12" s="47" t="str">
         <f aca="false">공수1!J4</f>
@@ -28853,7 +29533,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C13" s="47" t="str">
         <f aca="false">공수1!K4</f>
@@ -28929,7 +29609,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C14" s="47" t="str">
         <f aca="false">공수1!L4</f>
@@ -29005,7 +29685,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C15" s="47" t="str">
         <f aca="false">공수1!M4</f>
@@ -29081,7 +29761,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C16" s="47" t="str">
         <f aca="false">공수1!N4</f>
@@ -29157,7 +29837,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C17" s="47" t="str">
         <f aca="false">공수1!O4</f>
@@ -29233,7 +29913,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C18" s="47" t="str">
         <f aca="false">공수1!P4</f>
@@ -29309,7 +29989,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C19" s="47" t="str">
         <f aca="false">공수1!Q4</f>
@@ -29385,7 +30065,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C20" s="47" t="str">
         <f aca="false">공수1!R4</f>
@@ -29436,19 +30116,19 @@
         <v/>
       </c>
       <c r="O20" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P20" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q20" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R20" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S20" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29456,7 +30136,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C21" s="47" t="str">
         <f aca="false">공수1!S4</f>
@@ -29507,19 +30187,19 @@
         <v/>
       </c>
       <c r="O21" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P21" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q21" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R21" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S21" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29527,7 +30207,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C22" s="47" t="str">
         <f aca="false">공수1!T4</f>
@@ -29578,19 +30258,19 @@
         <v/>
       </c>
       <c r="O22" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P22" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q22" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R22" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S22" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29598,7 +30278,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C23" s="47" t="str">
         <f aca="false">공수1!U4</f>
@@ -29649,19 +30329,19 @@
         <v/>
       </c>
       <c r="O23" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P23" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q23" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R23" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S23" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29669,7 +30349,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C24" s="47" t="str">
         <f aca="false">공수1!V4</f>
@@ -29720,19 +30400,19 @@
         <v/>
       </c>
       <c r="O24" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P24" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q24" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R24" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S24" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29740,7 +30420,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C25" s="47" t="str">
         <f aca="false">공수1!W4</f>
@@ -29791,24 +30471,24 @@
         <v/>
       </c>
       <c r="O25" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P25" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q25" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R25" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S25" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="46" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="B28" s="46"/>
       <c r="C28" s="46"/>
@@ -29817,31 +30497,31 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="J29" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -29856,25 +30536,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="O29" s="24" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="P29" s="24" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="Q29" s="24" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="R29" s="24" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="S29" s="24" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29882,7 +30562,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C30" s="47" t="str">
         <f aca="false">공수2!D4</f>
@@ -29958,7 +30638,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C31" s="47" t="str">
         <f aca="false">공수2!E4</f>
@@ -30034,7 +30714,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C32" s="47" t="str">
         <f aca="false">공수2!F4</f>
@@ -30110,7 +30790,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C33" s="47" t="str">
         <f aca="false">공수2!G4</f>
@@ -30186,7 +30866,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C34" s="47" t="str">
         <f aca="false">공수2!H4</f>
@@ -30262,7 +30942,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C35" s="47" t="str">
         <f aca="false">공수2!I4</f>
@@ -30338,7 +31018,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C36" s="47" t="str">
         <f aca="false">공수2!J4</f>
@@ -30414,7 +31094,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C37" s="47" t="str">
         <f aca="false">공수2!K4</f>
@@ -30490,7 +31170,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C38" s="47" t="str">
         <f aca="false">공수2!L4</f>
@@ -30566,7 +31246,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C39" s="47" t="str">
         <f aca="false">공수2!M4</f>
@@ -30642,7 +31322,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C40" s="47" t="str">
         <f aca="false">공수2!N4</f>
@@ -30718,7 +31398,7 @@
         <v>12</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C41" s="47" t="str">
         <f aca="false">공수2!O4</f>
@@ -30794,7 +31474,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C42" s="47" t="str">
         <f aca="false">공수2!P4</f>
@@ -30870,7 +31550,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C43" s="47" t="str">
         <f aca="false">공수2!Q4</f>
@@ -30946,7 +31626,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C44" s="47" t="str">
         <f aca="false">공수2!R4</f>
@@ -30997,19 +31677,19 @@
         <v/>
       </c>
       <c r="O44" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P44" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q44" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R44" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S44" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31017,7 +31697,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C45" s="47" t="str">
         <f aca="false">공수2!S4</f>
@@ -31068,19 +31748,19 @@
         <v/>
       </c>
       <c r="O45" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P45" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q45" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R45" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S45" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31088,7 +31768,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C46" s="47" t="str">
         <f aca="false">공수2!T4</f>
@@ -31139,19 +31819,19 @@
         <v/>
       </c>
       <c r="O46" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P46" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q46" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R46" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S46" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31159,7 +31839,7 @@
         <v>18</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C47" s="47" t="str">
         <f aca="false">공수2!U4</f>
@@ -31210,19 +31890,19 @@
         <v/>
       </c>
       <c r="O47" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P47" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q47" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R47" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S47" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31230,7 +31910,7 @@
         <v>19</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C48" s="47" t="str">
         <f aca="false">공수2!V4</f>
@@ -31281,19 +31961,19 @@
         <v/>
       </c>
       <c r="O48" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P48" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q48" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R48" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S48" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31301,7 +31981,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C49" s="47" t="str">
         <f aca="false">공수2!W4</f>
@@ -31352,19 +32032,19 @@
         <v/>
       </c>
       <c r="O49" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="P49" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Q49" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="R49" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="S49" s="53" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make parent reports PDF-only and allow undecided advanced classes
- 선행 과목반 이름·소개를 비워 두고 나중에 엑셀에 입력하도록 변경
- 정하지 않은 반은 보고서에 '개별 상담을 통해 안내해 드립니다'로 표시
- 한글(HML) 보고서 생성 제거, 엑셀 기준 PDF 보고서만 생성

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="192">
   <si>
     <r>
       <rPr>
@@ -3251,106 +3251,6 @@
     <t xml:space="preserve">선행 과목반 이름</t>
   </si>
   <si>
-    <t xml:space="preserve">대수반</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지수와 로그</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지수함수와 로그함수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">삼각함수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수열을 선행하는 반으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공통수학을 마친 학생이 다음 단계로 나아가기 좋은 과정입니다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="9"/>
@@ -3358,7 +3258,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">← 실제 운영하는 선행반 이름</t>
+      <t xml:space="preserve">← 선행 과목반 이름</t>
     </r>
     <r>
       <rPr>
@@ -3377,7 +3277,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">소개로 수정</t>
+      <t xml:space="preserve">소개가 정해지면 입력</t>
     </r>
     <r>
       <rPr>
@@ -3387,7 +3287,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
@@ -3396,169 +3296,83 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">빈 줄에 추가 가능</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">미적분Ⅰ반</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">함수의 극한과 연속</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">예</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">미분</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">대수반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">적분을 선행하는 반으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">비어 있어도 보고서는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">대수 학습을 마친 학생에게 권장하는 과정입니다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">상담을 통해 안내</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">확률과 통계반</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">순열과 조합</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확률</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">통계를 선행하는 반으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공통수학의 경우의 수를 바탕으로 개념을 넓혀 가는 과정입니다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t xml:space="preserve">로 표시</t>
     </r>
   </si>
   <si>
@@ -7694,40 +7508,28 @@
       <c r="E63" s="4"/>
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="10" t="s">
+      <c r="A64" s="7"/>
+      <c r="B64" s="19"/>
+      <c r="C64" s="19"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="B64" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="C64" s="20"/>
-      <c r="D64" s="20"/>
-      <c r="E64" s="20"/>
-      <c r="F64" s="13" t="s">
-        <v>92</v>
-      </c>
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B65" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="C65" s="20"/>
-      <c r="D65" s="20"/>
-      <c r="E65" s="20"/>
+      <c r="A65" s="7"/>
+      <c r="B65" s="19"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B66" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
+      <c r="A66" s="7"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7"/>
@@ -7824,7 +7626,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7836,7 +7638,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7848,28 +7650,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7877,25 +7679,25 @@
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="H7" s="25" t="s">
         <v>107</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="H7" s="25" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8886,12 +8688,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -8921,7 +8723,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -8988,7 +8790,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -9079,7 +8881,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -9146,164 +8948,164 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="N5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="O5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="R5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="S5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="T5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="U5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="W5" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="X5" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="G5" s="14" t="s">
+      <c r="Y5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="Z5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="AA5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="M5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="N5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="O5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="P5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q5" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="R5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="S5" s="14" t="s">
+      <c r="AB5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="T5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="U5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="V5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="W5" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="X5" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="Y5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="AB5" s="30" t="s">
-        <v>127</v>
-      </c>
       <c r="AC5" s="30" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D6" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="J6" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="K6" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="L6" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="G6" s="31" t="s">
+      <c r="M6" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="N6" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="O6" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="J6" s="31" t="s">
+      <c r="P6" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="K6" s="31" t="s">
+      <c r="Q6" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="L6" s="31" t="s">
+      <c r="R6" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="M6" s="31" t="s">
+      <c r="S6" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="N6" s="31" t="s">
+      <c r="T6" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="O6" s="31" t="s">
+      <c r="U6" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="V6" s="32" t="s">
         <v>140</v>
       </c>
-      <c r="Q6" s="31" t="s">
+      <c r="W6" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="R6" s="32" t="s">
+      <c r="X6" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="S6" s="32" t="s">
+      <c r="Y6" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="T6" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="U6" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="V6" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="W6" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B19</f>
@@ -13902,10 +13704,6 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
-      <formula1>"하,중하,중,중상,상,최상"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="객관식은 1~5 사이 정수만 입력" errorStyle="stop" errorTitle="입력 오류" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:Q2 D7:Q86" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -13916,6 +13714,10 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:W4" type="list">
       <formula1>설정!$B$19:$B$22</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:W5" type="list">
+      <formula1>"하,중하,중,중상,상,최상"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -13948,12 +13750,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -13982,7 +13784,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -14049,7 +13851,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
@@ -14136,7 +13938,7 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -14203,161 +14005,161 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="N5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="O5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="R5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="S5" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="T5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="U5" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="W5" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="X5" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="G5" s="14" t="s">
+      <c r="Y5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="Z5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="AA5" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="M5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="N5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="O5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="P5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q5" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="R5" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="S5" s="14" t="s">
+      <c r="AB5" s="30" t="s">
         <v>121</v>
-      </c>
-      <c r="T5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="U5" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="V5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="W5" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="X5" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="Y5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA5" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="AB5" s="30" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D6" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="J6" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="K6" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="L6" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="G6" s="31" t="s">
+      <c r="M6" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="N6" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="O6" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="J6" s="31" t="s">
+      <c r="P6" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="K6" s="31" t="s">
+      <c r="Q6" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="L6" s="31" t="s">
+      <c r="R6" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="M6" s="31" t="s">
+      <c r="S6" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="N6" s="31" t="s">
+      <c r="T6" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="O6" s="31" t="s">
+      <c r="U6" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="V6" s="32" t="s">
         <v>140</v>
       </c>
-      <c r="Q6" s="31" t="s">
+      <c r="W6" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="R6" s="32" t="s">
+      <c r="X6" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="S6" s="32" t="s">
+      <c r="Y6" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="T6" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="U6" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="V6" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="W6" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="Z6" s="33" t="str">
         <f aca="false">설정!B24</f>
@@ -18687,7 +18489,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -18716,7 +18518,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -18745,78 +18547,78 @@
     </row>
     <row r="5" customFormat="false" ht="56.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="S5" s="3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E6" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="G6" s="4" t="s">
+      <c r="M6" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="N6" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="O6" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="P6" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="U6" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="V6" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="W6" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="P6" s="4" t="s">
+      <c r="X6" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="S6" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="T6" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="U6" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="V6" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="W6" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="Y6" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19399,7 +19201,7 @@
         <v/>
       </c>
       <c r="S13" s="5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
@@ -24123,7 +23925,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -24139,7 +23941,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -24155,40 +23957,40 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="L6" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28883,7 +28685,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -28905,7 +28707,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -28927,7 +28729,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="46" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B4" s="46"/>
       <c r="C4" s="46"/>
@@ -28936,31 +28738,31 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -28975,25 +28777,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="O5" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="P5" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q5" s="24" t="s">
+        <v>185</v>
+      </c>
+      <c r="R5" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="S5" s="24" t="s">
         <v>187</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="O5" s="24" t="s">
-        <v>189</v>
-      </c>
-      <c r="P5" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q5" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="R5" s="24" t="s">
-        <v>192</v>
-      </c>
-      <c r="S5" s="24" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29001,7 +28803,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C6" s="47" t="str">
         <f aca="false">공수1!D4</f>
@@ -29077,7 +28879,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C7" s="47" t="str">
         <f aca="false">공수1!E4</f>
@@ -29153,7 +28955,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C8" s="47" t="str">
         <f aca="false">공수1!F4</f>
@@ -29229,7 +29031,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C9" s="47" t="str">
         <f aca="false">공수1!G4</f>
@@ -29305,7 +29107,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C10" s="47" t="str">
         <f aca="false">공수1!H4</f>
@@ -29381,7 +29183,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C11" s="47" t="str">
         <f aca="false">공수1!I4</f>
@@ -29457,7 +29259,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C12" s="47" t="str">
         <f aca="false">공수1!J4</f>
@@ -29533,7 +29335,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C13" s="47" t="str">
         <f aca="false">공수1!K4</f>
@@ -29609,7 +29411,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C14" s="47" t="str">
         <f aca="false">공수1!L4</f>
@@ -29685,7 +29487,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C15" s="47" t="str">
         <f aca="false">공수1!M4</f>
@@ -29761,7 +29563,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C16" s="47" t="str">
         <f aca="false">공수1!N4</f>
@@ -29837,7 +29639,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C17" s="47" t="str">
         <f aca="false">공수1!O4</f>
@@ -29913,7 +29715,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C18" s="47" t="str">
         <f aca="false">공수1!P4</f>
@@ -29989,7 +29791,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C19" s="47" t="str">
         <f aca="false">공수1!Q4</f>
@@ -30065,7 +29867,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C20" s="47" t="str">
         <f aca="false">공수1!R4</f>
@@ -30116,19 +29918,19 @@
         <v/>
       </c>
       <c r="O20" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P20" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q20" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R20" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S20" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30136,7 +29938,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C21" s="47" t="str">
         <f aca="false">공수1!S4</f>
@@ -30187,19 +29989,19 @@
         <v/>
       </c>
       <c r="O21" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P21" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q21" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R21" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S21" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30207,7 +30009,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C22" s="47" t="str">
         <f aca="false">공수1!T4</f>
@@ -30258,19 +30060,19 @@
         <v/>
       </c>
       <c r="O22" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P22" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q22" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R22" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S22" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30278,7 +30080,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C23" s="47" t="str">
         <f aca="false">공수1!U4</f>
@@ -30329,19 +30131,19 @@
         <v/>
       </c>
       <c r="O23" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P23" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q23" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R23" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S23" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30349,7 +30151,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C24" s="47" t="str">
         <f aca="false">공수1!V4</f>
@@ -30400,19 +30202,19 @@
         <v/>
       </c>
       <c r="O24" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P24" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q24" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R24" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S24" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30420,7 +30222,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C25" s="47" t="str">
         <f aca="false">공수1!W4</f>
@@ -30471,24 +30273,24 @@
         <v/>
       </c>
       <c r="O25" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P25" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q25" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R25" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S25" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="46" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B28" s="46"/>
       <c r="C28" s="46"/>
@@ -30497,31 +30299,31 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J29" s="4" t="str">
         <f aca="false">설정!$B$6&amp;" 정답률"</f>
@@ -30536,25 +30338,25 @@
         <v>TF3반 정답률</v>
       </c>
       <c r="M29" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="N29" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="O29" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="P29" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q29" s="24" t="s">
+        <v>185</v>
+      </c>
+      <c r="R29" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="S29" s="24" t="s">
         <v>187</v>
-      </c>
-      <c r="N29" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="O29" s="24" t="s">
-        <v>189</v>
-      </c>
-      <c r="P29" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q29" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="R29" s="24" t="s">
-        <v>192</v>
-      </c>
-      <c r="S29" s="24" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30562,7 +30364,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C30" s="47" t="str">
         <f aca="false">공수2!D4</f>
@@ -30638,7 +30440,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C31" s="47" t="str">
         <f aca="false">공수2!E4</f>
@@ -30714,7 +30516,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C32" s="47" t="str">
         <f aca="false">공수2!F4</f>
@@ -30790,7 +30592,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C33" s="47" t="str">
         <f aca="false">공수2!G4</f>
@@ -30866,7 +30668,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C34" s="47" t="str">
         <f aca="false">공수2!H4</f>
@@ -30942,7 +30744,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C35" s="47" t="str">
         <f aca="false">공수2!I4</f>
@@ -31018,7 +30820,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C36" s="47" t="str">
         <f aca="false">공수2!J4</f>
@@ -31094,7 +30896,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C37" s="47" t="str">
         <f aca="false">공수2!K4</f>
@@ -31170,7 +30972,7 @@
         <v>9</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C38" s="47" t="str">
         <f aca="false">공수2!L4</f>
@@ -31246,7 +31048,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C39" s="47" t="str">
         <f aca="false">공수2!M4</f>
@@ -31322,7 +31124,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C40" s="47" t="str">
         <f aca="false">공수2!N4</f>
@@ -31398,7 +31200,7 @@
         <v>12</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C41" s="47" t="str">
         <f aca="false">공수2!O4</f>
@@ -31474,7 +31276,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C42" s="47" t="str">
         <f aca="false">공수2!P4</f>
@@ -31550,7 +31352,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C43" s="47" t="str">
         <f aca="false">공수2!Q4</f>
@@ -31626,7 +31428,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C44" s="47" t="str">
         <f aca="false">공수2!R4</f>
@@ -31677,19 +31479,19 @@
         <v/>
       </c>
       <c r="O44" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P44" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q44" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R44" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S44" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31697,7 +31499,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C45" s="47" t="str">
         <f aca="false">공수2!S4</f>
@@ -31748,19 +31550,19 @@
         <v/>
       </c>
       <c r="O45" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P45" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q45" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R45" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S45" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31768,7 +31570,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C46" s="47" t="str">
         <f aca="false">공수2!T4</f>
@@ -31819,19 +31621,19 @@
         <v/>
       </c>
       <c r="O46" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P46" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q46" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R46" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S46" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31839,7 +31641,7 @@
         <v>18</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C47" s="47" t="str">
         <f aca="false">공수2!U4</f>
@@ -31890,19 +31692,19 @@
         <v/>
       </c>
       <c r="O47" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P47" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q47" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R47" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S47" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31910,7 +31712,7 @@
         <v>19</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C48" s="47" t="str">
         <f aca="false">공수2!V4</f>
@@ -31961,19 +31763,19 @@
         <v/>
       </c>
       <c r="O48" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P48" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q48" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R48" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S48" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31981,7 +31783,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C49" s="47" t="str">
         <f aca="false">공수2!W4</f>
@@ -32032,19 +31834,19 @@
         <v/>
       </c>
       <c r="O49" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="P49" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Q49" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="R49" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="S49" s="53" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace matrix problems 6 and 9 in 공통수학1 (9 uses powers of a complex number)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Etsous4c5JTLk1TXqQRtGW
</commit_message>
<xml_diff>
--- a/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
+++ b/반편성고사/예비고1_반편성고사_채점_반배정.xlsx
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I4" s="21" t="inlineStr">
         <is>
-          <t>행렬</t>
+          <t>경우의 수</t>
         </is>
       </c>
       <c r="J4" s="21" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="L4" s="21" t="inlineStr">
         <is>
-          <t>행렬</t>
+          <t>방정식과 부등식</t>
         </is>
       </c>
       <c r="M4" s="21" t="inlineStr">

</xml_diff>